<commit_message>
Adding DAY47/ DAY48/ DAY49/ DAY50/ DAY51/ WEBDESIGN
</commit_message>
<xml_diff>
--- a/CU-.NET-Batch4-Assignments-Repositories.xlsx
+++ b/CU-.NET-Batch4-Assignments-Repositories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sahil\study material\SEM-8\CAPGEMINI\CU-DotNet-Jan26-B4\CU-DotNet-Jan26-B4-Sahil-Ittan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5683628D-99B6-4CA6-9EDB-C563D91CF1CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3F01C4-BE9C-443D-9A7F-44E98C0FD385}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C99DFE55-A9F3-4CE7-8732-71313EE2B406}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="49">
   <si>
     <t>SNO</t>
   </si>
@@ -163,13 +163,31 @@
   </si>
   <si>
     <t>Day10-01 Methods Orders.docx</t>
+  </si>
+  <si>
+    <t>https://github.com/Jamiwal-3704/CU-DotNet-Jan26-B4-Sahil-Ittan/tree/main/DAY3</t>
+  </si>
+  <si>
+    <t>https://github.com/Jamiwal-3704/CU-DotNet-Jan26-B4-Sahil-Ittan/blob/main/Day2_ValueTypes_Conversions_Exercises.pdf</t>
+  </si>
+  <si>
+    <t>https://github.com/Jamiwal-3704/CU-DotNet-Jan26-B4-Sahil-Ittan/tree/main/DAY4</t>
+  </si>
+  <si>
+    <t>https://github.com/Jamiwal-3704/CU-DotNet-Jan26-B4-Sahil-Ittan/tree/main/DAY5</t>
+  </si>
+  <si>
+    <t>https://github.com/Jamiwal-3709/CU-DotNth-Jan26-B9-Sahil-Ittan/tree/main/DAY10</t>
+  </si>
+  <si>
+    <t>https://github.com/Jamiwal-3704/CU-DotNet-Jan26-B4-Sahil-Ittan/tree/main/DAY6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,6 +205,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -209,17 +235,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -566,6 +595,9 @@
       <c r="B2" t="s">
         <v>34</v>
       </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
@@ -574,6 +606,9 @@
       <c r="B3" t="s">
         <v>35</v>
       </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
@@ -582,6 +617,9 @@
       <c r="B4" t="s">
         <v>36</v>
       </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
@@ -590,6 +628,9 @@
       <c r="B5" t="s">
         <v>37</v>
       </c>
+      <c r="C5" s="3" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
@@ -598,6 +639,9 @@
       <c r="B6" t="s">
         <v>38</v>
       </c>
+      <c r="C6" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
@@ -875,6 +919,10 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{CAA485DE-332F-4A15-B80A-E2CB306430DA}"/>
+    <hyperlink ref="C6" r:id="rId2" xr:uid="{072DB743-796A-429B-B940-AEEDDACB3DA1}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>